<commit_message>
Default currency and proxy
</commit_message>
<xml_diff>
--- a/public/tests/data/test_simple.xlsx
+++ b/public/tests/data/test_simple.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\github\jonaskello\backcel\public\tests\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6646896-9B02-44A9-9632-24DC20A72B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CF7A474-E95D-4749-8487-C10811C735FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="38">
   <si>
     <t>Name</t>
   </si>
@@ -87,12 +87,6 @@
   </si>
   <si>
     <t>Portfolios</t>
-  </si>
-  <si>
-    <t>Currency</t>
-  </si>
-  <si>
-    <t>Proxy</t>
   </si>
   <si>
     <t>Date</t>
@@ -577,13 +571,13 @@
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
@@ -616,46 +610,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C271D88-DDEC-4A65-8905-A99CA73725FC}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" width="14.921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -673,7 +655,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>10</v>
@@ -1050,16 +1032,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>18</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="7" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.4">
@@ -1525,24 +1507,24 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>20</v>
-      </c>
       <c r="E1" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B2" s="4" t="s">
         <v>10</v>
@@ -2188,46 +2170,46 @@
     <row r="1" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="I1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="J1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="M1" s="1" t="s">
         <v>32</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="N1" s="1"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B2" s="2">
         <v>45658</v>
@@ -2236,10 +2218,10 @@
         <v>45689</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F2" s="5">
         <v>31</v>
@@ -2254,7 +2236,7 @@
         <v>79.53</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="K2" s="5">
         <v>0</v>
@@ -2263,12 +2245,12 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="2">
         <v>45658</v>
@@ -2277,10 +2259,10 @@
         <v>45689</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F3" s="5">
         <v>-10</v>
@@ -2304,12 +2286,12 @@
         <v>-10</v>
       </c>
       <c r="M3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2">
         <v>45658</v>
@@ -2318,10 +2300,10 @@
         <v>45689</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="F4" s="5">
         <v>10.5</v>
@@ -2345,7 +2327,7 @@
         <v>-4.1900000000000004</v>
       </c>
       <c r="M4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>